<commit_message>
Fix: - Quản lý Đê/Kè - [F-160] Biểu 13-N: Thống kê về hệ thống đê, kè chắn sóng, chắn cát - Cho phép Hệ thống VTS, Trạm Radar, Đê/kè vẫn có thể chỉnh sửa sau khi đã phê duyệt
</commit_message>
<xml_diff>
--- a/src/main/resources/public/template_export/BCKCHT_175.xlsx
+++ b/src/main/resources/public/template_export/BCKCHT_175.xlsx
@@ -166,19 +166,19 @@
     <t>${item.caoTrinhDinh.asText()}</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',item.hienTrang.asText(), 'TINH_TRANG')}</t>
-  </si>
-  <si>
-    <t>${thiz.getCateOtherText('DM_APP_PARAM',item.loaiCongTrinh.asText(), 'LOAI_KCCT_DE_KE')}</t>
-  </si>
-  <si>
     <t>${fkDonViBcText}</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('AUTH_ORG',item.donViQuanLy.asText())}</t>
-  </si>
-  <si>
-    <t>${thiz.getCateOtherText('DM_DON_VI_HANH_CHINH',item.viTriDiaDanh.asText())}</t>
+    <t>${this.getCateOtherText('DM_APP_PARAM',item.loaiCongTrinh.asText(), 'LOAI_KCCT_DE_KE')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_DON_VI_HANH_CHINH',item.viTriDiaDanh.asText())}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('DM_APP_PARAM',item.hienTrang.asText(), 'TINH_TRANG')}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('AUTH_ORG',item.donViQuanLy.asText())}</t>
   </si>
 </sst>
 </file>
@@ -404,8 +404,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -413,18 +422,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -441,6 +438,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -722,12 +722,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J17"/>
-  <sheetFormatPr defaultRowHeight="15" ns2:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -739,52 +739,52 @@
     <col min="10" max="10" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="14"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="17"/>
-    </row>
-    <row r="2" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="J1" s="14"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="22"/>
+      <c r="B2" s="21"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="18"/>
-    </row>
-    <row r="3" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="I2" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" s="15"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="22"/>
+      <c r="B3" s="21"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" ns2:dyDescent="0.25">
+      <c r="J3" s="14"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -792,12 +792,12 @@
       <c r="E4" s="5"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
-      <c r="I4" s="18" t="s">
+      <c r="I4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="18"/>
-    </row>
-    <row r="5" spans="1:10" ns2:dyDescent="0.25">
+      <c r="J4" s="15"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -808,80 +808,80 @@
       <c r="H5" s="5"/>
       <c r="J5" s="6"/>
     </row>
-    <row r="6" spans="1:10" ht="15.75" ns2:dyDescent="0.25">
-      <c r="A6" s="23" t="s">
+    <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-    </row>
-    <row r="7" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A7" s="24" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-    </row>
-    <row r="8" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-    </row>
-    <row r="9" spans="1:10" ht="15" customHeight="1" ns2:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
+    </row>
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="13" t="s">
+      <c r="G9" s="19"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="16" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="45" customHeight="1" ns2:dyDescent="0.25">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
+    <row r="10" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
       <c r="F10" s="1" t="s">
         <v>19</v>
       </c>
@@ -891,10 +891,10 @@
       <c r="H10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" customHeight="1" ns2:dyDescent="0.25">
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1">
         <v>1</v>
@@ -924,7 +924,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="19.5" customHeight="1" ns2:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>11</v>
       </c>
@@ -935,7 +935,7 @@
         <v>30</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>25</v>
@@ -950,13 +950,13 @@
         <v>28</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ns2:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -968,54 +968,60 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
       <c r="D14" s="8"/>
       <c r="E14" s="5"/>
       <c r="G14" s="8"/>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-    </row>
-    <row r="15" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
       <c r="D15" s="8"/>
       <c r="E15" s="5"/>
       <c r="G15" s="8"/>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-    </row>
-    <row r="16" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-    </row>
-    <row r="17" spans="1:10" ns2:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
     <mergeCell ref="A15:C17"/>
     <mergeCell ref="H14:J14"/>
     <mergeCell ref="H15:J17"/>
@@ -1032,15 +1038,9 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" fitToWidth="1" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="3" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>